<commit_message>
day 6 cpmpleted data cleaning in excel and filehandling
</commit_message>
<xml_diff>
--- a/excel/student_data_cleaning.xlsx
+++ b/excel/student_data_cleaning.xlsx
@@ -8,13 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data_analyst_journey2026\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{5E5FD6DA-A22D-4235-8894-321F099A5606}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{447E29B1-FB4C-475D-BC44-FC30A7427C16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{63FE48FE-9EFC-4FF4-B081-EC181C94C198}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sheet1!$A$1:$C$9</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
@@ -33,10 +36,76 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="15">
+  <si>
+    <t>Student</t>
+  </si>
+  <si>
+    <t>Department</t>
+  </si>
+  <si>
+    <t>Marks</t>
+  </si>
+  <si>
+    <t>Abhi</t>
+  </si>
+  <si>
+    <t>AIML</t>
+  </si>
+  <si>
+    <t>Sai</t>
+  </si>
+  <si>
+    <t>Ravi</t>
+  </si>
+  <si>
+    <t>CSE</t>
+  </si>
+  <si>
+    <t>Kiran</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>Mohan</t>
+  </si>
+  <si>
+    <t>EEE</t>
+  </si>
+  <si>
+    <t>ECE</t>
+  </si>
+  <si>
+    <t>Arjun</t>
+  </si>
+  <si>
+    <t>Teja</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -64,13 +133,42 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="0"/>
+  <dxfs count="1">
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+  </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -380,9 +478,118 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{87D3952E-BC72-4F07-8BD6-2535748AA619}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="13.44140625" customWidth="1"/>
+    <col min="2" max="2" width="18.5546875" customWidth="1"/>
+    <col min="3" max="3" width="19.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
+        <v>13</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" s="2">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B3" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" s="2">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="4" t="s">
+        <v>6</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="2">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="6"/>
+      <c r="B5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="C5" s="2">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" s="2">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="C7" s="2">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="5"/>
+    </row>
+  </sheetData>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C9">
+    <sortCondition descending="1" ref="C2:C9"/>
+  </sortState>
+  <conditionalFormatting sqref="C2:C8">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="greaterThan">
+      <formula>90</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>